<commit_message>
🔧 Corrección de oficina: SABINAS HIDALGO
</commit_message>
<xml_diff>
--- a/public/CLAVES_ETRANSPORTE/OFICINAS NOMENCLATURAS.xlsx
+++ b/public/CLAVES_ETRANSPORTE/OFICINAS NOMENCLATURAS.xlsx
@@ -1384,8 +1384,8 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71">
-        <v>93</v>
+      <c r="A71" t="str">
+        <v>0093</v>
       </c>
       <c r="B71" t="str">
         <v>SABINAS HIDALGO</v>

</xml_diff>

<commit_message>
🔧 Corrección de oficina: LAGOS DE MORENO
</commit_message>
<xml_diff>
--- a/public/CLAVES_ETRANSPORTE/OFICINAS NOMENCLATURAS.xlsx
+++ b/public/CLAVES_ETRANSPORTE/OFICINAS NOMENCLATURAS.xlsx
@@ -740,8 +740,8 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25">
-        <v>31</v>
+      <c r="A25" t="str">
+        <v>0031</v>
       </c>
       <c r="B25" t="str">
         <v>LAGOS DE MORENO</v>

</xml_diff>